<commit_message>
feat: Aux Timer column in downloadable template + required-columns callout
- rebuild showflow-template.xlsx: Aux Timer column (amber header, hover
  instructions, sample reset rows) between Colour and the custom fields;
  Timer Type kept with none/count-down for the primary timer and a note
  that the column may be dropped (colour fallback); sample data fixed so
  the template parses with zero warnings
- add script/generate-template.py so the template is reproducible
- settings dialog: Aux Timer callout under the 8 required columns;
  Timer Type hint mentions the colour fallback
- README: template section covers Aux Timer + regeneration
- v2.3.2
</commit_message>
<xml_diff>
--- a/client/public/showflow-template.xlsx
+++ b/client/public/showflow-template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,24 +29,20 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
-      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B45309"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,7 +85,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -92,31 +93,28 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="00D0D0D0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -241,9 +239,11 @@
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>REQUIRED
+        <t>REQUIRED (may be omitted entirely)
+Controls the item's primary timer in Ontime:
 none        = no countdown timer for this item
-count-down  = show a countdown timer (typical for speaker segments)</t>
+count-down  = show a countdown timer (typical for speaker segments)
+If you delete this whole column, the timer type is inferred from Colour instead: Blue → count-down, everything else → none.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -255,41 +255,50 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
+        <t>OPTIONAL — special column (NOT a custom field).
+Drives Ontime's Aux timer 1 with automations built at sync time.
+Put a duration (e.g. 1:00:00 or 0:40:00) on the row where the aux timer should reset and start counting down. It keeps running across items until another row resets it, and it stops when you stop the show.
+Leave cells blank or write "none" on rows that don't touch it — or delete the whole column if you don't use aux timers.
+Keep Aux timer 1 set to count-down direction in Ontime.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
         <t>OPTIONAL — becomes a custom field in Ontime.
 Which screen look is live, e.g. SS1 / SS2 / SS3.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>OPTIONAL — becomes a custom field in Ontime.
 Video cue for this item, e.g. "Roll opener video".</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>OPTIONAL — becomes a custom field in Ontime.
 Lighting cue, e.g. "Stage wash", "House to half".</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>OPTIONAL — becomes a custom field in Ontime.
 Audio cue, e.g. "Podium mic live", "Play walk-in music".</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>OPTIONAL — becomes a custom field in Ontime.
 Who is on stage / at the podium.</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>OPTIONAL — becomes a custom field in Ontime.
 Stage action, e.g. "Lectern on", "Panel chairs set".</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>OPTIONAL
 Free-form production notes (goes to the Ontime note field, not a custom field).
@@ -589,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -600,13 +609,14 @@
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -652,70 +662,75 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
+          <t>Aux Timer</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
           <t>Screenstate</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Lighting</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Audio</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Speakers</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>0:30:00</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Walk-in — doors open</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
@@ -725,56 +740,52 @@
           <t>Green</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>SS1</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>House look</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Walk-in music</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr"/>
-      <c r="N2" s="3" t="inlineStr"/>
-      <c r="O2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>0:01:30</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0:01:00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>9:31 AM</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Opener video</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>none</t>
         </is>
@@ -784,64 +795,62 @@
           <t>Yellow</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>SS1</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Roll opener video</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Stage dark</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Video audio full</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Video from client</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>9:31 AM</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>0:02:00</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>9:33 AM</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>MC intro</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
@@ -851,64 +860,62 @@
           <t>Purple</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>SS2</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Stage wash</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Podium mic live</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>MC</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>MC walks from SR</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>9:33 AM</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>0:25:00</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>9:58 AM</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>CEO Welcome + PPT</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>count-down</t>
         </is>
@@ -918,72 +925,77 @@
           <t>Blue</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1:00:00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>SS3</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Advance PPT</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Podium special</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Podium mic</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Lectern on</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>Confidence monitor shows timer</t>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Aux resets to 1h here and counts down</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>9:58 AM</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>0:02:00</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>MC outro to break</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>none</t>
         </is>
@@ -993,60 +1005,62 @@
           <t>Purple</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>SS2</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Stage wash</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Podium mic live</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>MC</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr"/>
-      <c r="O6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>0:15:00</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>10:15 AM</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Break</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>none</t>
         </is>
@@ -1056,27 +1070,29 @@
           <t>Green</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0:15:00</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>SS1</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>House look</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Break music</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr"/>
-      <c r="N7" s="3" t="inlineStr"/>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>Pinned — break always starts at 10:00</t>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Pinned — break always starts at 10:00 · aux resets to 15 min</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1105,127 +1121,141 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr"/>
-    </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>1.  Keep the first eight columns exactly as named — they are required:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">     Cue #, Start Time, Duration, End Time, Linkstart, Title, Timer Type, Colour</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr"/>
-    </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>2.  Linkstart controls timing:</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">     TRUE  → the item starts when the previous one ends (rolls with the show)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">     FALSE → the item is pinned to the clock time in Start Time (doors, breaks, hard outs)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>3.  Timer Type: 'count-down' shows a countdown timer in Ontime, 'none' does not.</t>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>3.  Timer Type drives each item's primary timer: 'count-down' shows a countdown in Ontime, 'none' does not.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>4.  Colour must be Yellow, Green, Purple or Blue:</t>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     You may delete the whole column — the timer type is then inferred from Colour (Blue → count-down, others → none).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>4.  Colour must be Yellow, Green, Purple or Blue:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">     Yellow = videos · Green = breaks / walk-ins · Purple = intros / outros · Blue = speaking segments</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>5.  Every column you add after the required eight becomes an Ontime custom field automatically</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">     (Screenstate, Video, Lighting, Audio, Speakers, Stage are just examples — rename or add your own).</t>
+          <t>5.  Aux Timer (optional, special): drives Ontime's Aux timer 1 via automations created at sync time.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     'Notes' is special: it fills the Ontime note field instead.</t>
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Put a duration (e.g. 1:00:00) on the row where the aux timer should reset and start counting down.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr"/>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     It keeps running across items until another row resets it, and it stops when you stop the show.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>6.  Upload this file to Google Sheets (File → Import), then paste the sheet ID and tab name</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+          <t xml:space="preserve">     Blank or 'none' on rows that don't touch it. Delete the column if you don't use aux timers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>6.  Every other column you add after the required eight becomes an Ontime custom field automatically</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     (Screenstate, Video, Lighting, Audio, Speakers, Stage are just examples — rename or add your own).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     'Notes' is special: it fills the Ontime note field instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>7.  Upload this file to Google Sheets (File → Import), then paste the sheet ID and tab name</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">     into the tool's Settings (gear icon).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Hover over any header cell on the 'Show Flow' tab for details on that column.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Technical support: mosc-tools@moscone.ca</t>
         </is>

</xml_diff>

<commit_message>
v2.4.0: Aux Timer 00:00:00 clears the timer
An explicit 00:00:00 in the Aux Timer column now builds a clear
automation: on that cue's start, Aux 1 stops and is set to 00:00:00
(no restart), so aux displays show nothing until the next reset row.
Previously a zero value was silently ignored.

- parse: 0 kept as clear marker (blank/'none' still null); no
  under-a-minute warning for explicit zero; clearer no-cue warning
- buildAuxAutomations: clear rows emit stop->set(00:00:00) only,
  titled 'Mosc-sync aux: cue N -> clear'; UI cue list shows 'clear'
- template hover text + How-it-works sheet, dashboard callout, README
- QA: clear-row assertions added (fixture now 8 rows)
</commit_message>
<xml_diff>
--- a/client/public/showflow-template.xlsx
+++ b/client/public/showflow-template.xlsx
@@ -258,6 +258,7 @@
         <t>OPTIONAL — special column (NOT a custom field).
 Drives Ontime's Aux timer 1 with automations built at sync time.
 Put a duration (e.g. 1:00:00 or 0:40:00) on the row where the aux timer should reset and start counting down. It keeps running across items until another row resets it, and it stops when you stop the show.
+00:00:00 clears the timer: it stops, zeroes out, and displays show nothing until the next reset row.
 Leave cells blank or write "none" on rows that don't touch it — or delete the whole column if you don't use aux timers.
 Keep Aux timer 1 set to count-down direction in Ontime.</t>
       </text>
@@ -1208,6 +1209,13 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">     00:00:00 clears the timer — it stops, zeroes out, and displays show nothing until the next reset row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">     Blank or 'none' on rows that don't touch it. Delete the column if you don't use aux timers.</t>
         </is>
       </c>

</xml_diff>